<commit_message>
version 54 - Update Test validation, using RAGAS and run several times
</commit_message>
<xml_diff>
--- a/FastAPI_AI_Service/app/Chunking/report_data_for_classification.xlsx
+++ b/FastAPI_AI_Service/app/Chunking/report_data_for_classification.xlsx
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Candles_Knowledge\Some_Fragrance_layers_of_scented_candles.docx</t>
+          <t>Some_Fragrance_layers_of_scented_candles.docx</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -469,7 +469,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Candles_Knowledge\Some_Fragrance_layers_of_scented_candles.docx</t>
+          <t>Some_Fragrance_layers_of_scented_candles.docx</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -491,7 +491,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Candles_Knowledge\Some_Fragrance_layers_of_scented_candles.docx</t>
+          <t>Some_Fragrance_layers_of_scented_candles.docx</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -513,7 +513,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Candles_Knowledge\Candle_benefit.docx</t>
+          <t>Candle_benefit.docx</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Candles_Knowledge\Candle_benefit.docx</t>
+          <t>Candle_benefit.docx</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Candles_Knowledge\Candle_benefit.docx</t>
+          <t>Candle_benefit.docx</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -579,7 +579,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Candles_Knowledge\Candle_benefit.docx</t>
+          <t>Candle_benefit.docx</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Discount_program\coupons.csv</t>
+          <t>coupons.csv</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Discount_program\coupons.csv</t>
+          <t>coupons.csv</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Discount_program\coupons.csv</t>
+          <t>coupons.csv</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Discount_program\coupons.csv</t>
+          <t>coupons.csv</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Discount_program\coupons.csv</t>
+          <t>coupons.csv</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\User_guidance\Safe_Usage_guidance.docx</t>
+          <t>Safe_Usage_guidance.docx</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\User_guidance\Safe_Usage_guidance.docx</t>
+          <t>Safe_Usage_guidance.docx</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Policies\Chinh_sach_mua_hang.docx</t>
+          <t>Chinh_sach_mua_hang.docx</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Policies\Chinh_sach_mua_hang.docx</t>
+          <t>Chinh_sach_mua_hang.docx</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -3240,7 +3240,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Policies\Chinh_sach_mua_hang.docx</t>
+          <t>Chinh_sach_mua_hang.docx</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Policies\Chinh_sach_mua_hang.docx</t>
+          <t>Chinh_sach_mua_hang.docx</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Policies\Chinh_sach_mua_hang.docx</t>
+          <t>Chinh_sach_mua_hang.docx</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Policies\Chinh_sach_mua_hang.docx</t>
+          <t>Chinh_sach_mua_hang.docx</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Policies\Chinh_sach_mua_hang.docx</t>
+          <t>Chinh_sach_mua_hang.docx</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Policies\Chinh_sach_mua_hang.docx</t>
+          <t>Chinh_sach_mua_hang.docx</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Policies\Chinh_sach_mua_hang.docx</t>
+          <t>Chinh_sach_mua_hang.docx</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Policies\Chinh_sach_mua_hang.docx</t>
+          <t>Chinh_sach_mua_hang.docx</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Common_FAQ.md</t>
+          <t>Common_FAQ.md</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -4278,7 +4278,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\3_Day_WKND.md</t>
+          <t>3_Day_WKND.md</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Amber_And_Vanilla.md</t>
+          <t>Amber_And_Vanilla.md</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\BLOW_A_WISH.md</t>
+          <t>BLOW_A_WISH.md</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -4374,7 +4374,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Candle_holder.md</t>
+          <t>Candle_holder.md</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -4406,7 +4406,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Candle_matchbox.md</t>
+          <t>Candle_matchbox.md</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Candle_metal_tray.md</t>
+          <t>Candle_metal_tray.md</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -4470,7 +4470,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Candle_pinwheel.md</t>
+          <t>Candle_pinwheel.md</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -4502,7 +4502,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Candle_rotation_tray.md</t>
+          <t>Candle_rotation_tray.md</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -4534,7 +4534,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Candle_Scissor.md</t>
+          <t>Candle_Scissor.md</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -4566,7 +4566,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Candle_Snuffer.md</t>
+          <t>Candle_Snuffer.md</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -4598,7 +4598,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Candle_Tray.md</t>
+          <t>Candle_Tray.md</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Coconut_And_Sea_Salt.md</t>
+          <t>Coconut_And_Sea_Salt.md</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -4662,7 +4662,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Dalat_Gift.md</t>
+          <t>Dalat_Gift.md</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -4694,7 +4694,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Day_Party.md</t>
+          <t>Day_Party.md</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Jasmin_ylang_ylang_sandalwood.md</t>
+          <t>Jasmin_ylang_ylang_sandalwood.md</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Lavander_Vanilia.md</t>
+          <t>Lavander_Vanilia.md</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Lumos_And_Cucumber.md</t>
+          <t>Lumos_And_Cucumber.md</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Lumos_Cajeput.md</t>
+          <t>Lumos_Cajeput.md</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -4854,7 +4854,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Lumos_cold.md</t>
+          <t>Lumos_cold.md</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Lumos_Honeydrew_And_Coconut.md</t>
+          <t>Lumos_Honeydrew_And_Coconut.md</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Lumos_Juicy_Peach.md</t>
+          <t>Lumos_Juicy_Peach.md</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -4950,7 +4950,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Lumos_Lemongrass.md</t>
+          <t>Lumos_Lemongrass.md</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -4982,7 +4982,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Lumos_menthol.md</t>
+          <t>Lumos_menthol.md</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Lumos_Midnight_sandalwood.md</t>
+          <t>Lumos_Midnight_sandalwood.md</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -5046,7 +5046,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Lumos_Rose_Boutique.md</t>
+          <t>Lumos_Rose_Boutique.md</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -5078,7 +5078,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Lumos_Tropical_Orchard.md</t>
+          <t>Lumos_Tropical_Orchard.md</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -5110,7 +5110,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Milk_Vanilla.md</t>
+          <t>Milk_Vanilla.md</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -5142,7 +5142,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Nen_and_Hoa.md</t>
+          <t>Nen_and_Hoa.md</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -5174,7 +5174,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Sandalwood_And_Rose.md</t>
+          <t>Sandalwood_And_Rose.md</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Shower_Playlist.md</t>
+          <t>Shower_Playlist.md</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -5238,7 +5238,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\smells_like_cacao_and_vanilla.md</t>
+          <t>smells_like_cacao_and_vanilla.md</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Sunset_Disco.md</t>
+          <t>Sunset_Disco.md</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Warn_Cider_And_Cinamon.md</t>
+          <t>Warn_Cider_And_Cinamon.md</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\Wood_tray.md</t>
+          <t>Wood_tray.md</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>D:\Website_NenThomBnC\Website_NenThomBnC\FastAPI_AI_Service\app\data\NenThom_data\Product_Catalogs\YOU_ARE_THE_MAGIC.md</t>
+          <t>YOU_ARE_THE_MAGIC.md</t>
         </is>
       </c>
       <c r="C221" t="n">

</xml_diff>